<commit_message>
Leads: 2026-10-15 04:12 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-15.xlsx
+++ b/output/leads_2026-10-15.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Air Necessities</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>theairnecessities.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.theairnecessities.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Air Necessities</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>admin@theairnecessities.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>830-652-1900</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>88</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>AC installation New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-15 13:19 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-15.xlsx
+++ b/output/leads_2026-10-15.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,62 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Emergency &amp; Residential Plumbing in Denton County, TX</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>steadfastplumbingtx.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.steadfastplumbingtx.com/sewar-repair-tx</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>joey@steadfastplumbingtx.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>817.368.0824</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Denton TX</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>sewer repair Denton TX</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-15 13:25 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-15.xlsx
+++ b/output/leads_2026-10-15.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -704,7 +704,6 @@
           <t>https://www.steadfastplumbingtx.com/sewar-repair-tx</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>joey@steadfastplumbingtx.com</t>
@@ -734,6 +733,126 @@
         </is>
       </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>compacthvac</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>compacthvac.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.compacthvac.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Alfred Castro</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nycompacthvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>845-222-2800</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>New York NY</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>HVAC contractor New York NY</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Atlantic Mechanical LLC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>atlantichvac.us</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://atlantichvac.us/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>nick@atlantichvac.us</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(917) 702-1748</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>New York NY</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>HVAC contractor New York NY</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-15 13:29 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-15.xlsx
+++ b/output/leads_2026-10-15.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -858,6 +858,126 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>John the Plumber</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>johntheplumberkansascity.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://johntheplumberkansascity.com/water-heater-installation-repair/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Kansas City</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>contact@johntheplumberkansascity.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(816) 708-2020</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Kansas City KS</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>water heater repair Kansas City KS</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Roof Ohio</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>roof-ohio.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://roof-ohio.com/locations-we-serve/columbus/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Armed Forces</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>info@roof-ohio.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(614) 741-3333</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Columbus OH</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roof repair company Columbus OH</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-15 19:53 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-15.xlsx
+++ b/output/leads_2026-10-15.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,178 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Brotherhood Roofing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>brotherhoodroofing.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://brotherhoodroofing.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@brotherhoodroofing.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>972-742-5332</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofer Frisco TX</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Phoenix Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>phoenixairca.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://phoenixairca.com/city/irvine-ca/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>holly@phoenixairca.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>949-481-0204</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Irvine CA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>HVAC contractor Irvine CA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Catalyst Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>catalystroofingsiding.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://catalystroofingsiding.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Roof Quote</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>colton@catalystroofingsiding.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(260) 633-4031</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>78</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>roofing contractor Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-15 20:09 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-15.xlsx
+++ b/output/leads_2026-10-15.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -999,7 +999,6 @@
           <t>https://brotherhoodroofing.com/</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>info@brotherhoodroofing.com</t>
@@ -1055,7 +1054,6 @@
           <t>https://phoenixairca.com/city/irvine-ca/</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>holly@phoenixairca.com</t>
@@ -1145,6 +1143,122 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Same Day San Diego</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>samedaysd.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://samedaysd.com/locations/escondido/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Jonathan Wintersteller</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@samedaysd.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(619) 762-3044</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Escondido CA</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>heat pump installation Escondido CA</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ElectrifyCalc</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>electrifycalc.site</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.electrifycalc.site/guides/heat-pump-installation-cost-california-2026</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Editorial Team</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>info@electrifycalc.site</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Escondido CA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>70</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>heat pump installation Escondido CA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-15 22:34 UTC (cycle 115)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-15.xlsx
+++ b/output/leads_2026-10-15.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1239,7 +1239,6 @@
           <t>info@electrifycalc.site</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Escondido CA</t>
@@ -1259,6 +1258,122 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Albi Air Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>albiair.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://albiair.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>albihvac@albiair.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(479) 530-9406</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>HVAC contractor Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Royal Flush Plumbing</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>royalflushplumb.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.royalflushplumb.com/services/sewer-repair</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>King County</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>meghan@royalflushplumb.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(253) 366-2904</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Tacoma WA</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>sewer repair Tacoma WA</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-15 22:36 UTC (cycle 116)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-15.xlsx
+++ b/output/leads_2026-10-15.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1284,7 +1284,6 @@
           <t>https://albiair.com/</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>albihvac@albiair.com</t>
@@ -1374,6 +1373,126 @@
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>T Rock Roofing &amp; Contracting - Dallas-Fort Worth Trusted Roofer</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>dallasroofer.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://dallasroofer.com/mckinney/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@dallasroofer.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>469.931.9867</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>roofer McKinney TX</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HVAC Plus LLC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>hvacplususa.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.hvacplususa.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Middle Tennessee</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>hvacplus28@gmail.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>615-955-4660</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>98</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>HVAC contractor Nashville TN</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>

</xml_diff>